<commit_message>
Latest generated outputs 2026-03-10
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/advertising-advertising.xlsx
+++ b/generated/spreadsheet/advertising-advertising.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -568,14 +568,14 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Application sub type</t>
+          <t>Planning authority</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Further classification of the application type for specific variations within the main application type</t>
+          <t>A reference of the planning authority the application has been submitted to, e.g. local-authority:CMD for London borough of Camden</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -599,19 +599,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Planning authority</t>
+          <t>Submission date</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>A reference of the planning authority the application has been submitted to, e.g. local-authority:CMD for London borough of Camden</t>
+          <t>Date the application is submitted in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -630,19 +630,19 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Submission date</t>
+          <t>Modules[]</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Date the application is submitted in YYYY-MM-DD format</t>
+          <t>List of required modules for this application that can be used to validate the application</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -661,14 +661,18 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Modules[]</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>Documents[]</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>List of required modules for this application that can be used to validate the application</t>
+          <t>Unique reference for the document within this application submission, generated by the submitting system</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -697,13 +701,13 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Unique reference for the document within this application submission, generated by the submitting system</t>
+          <t>The name or title of the document</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -732,13 +736,13 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>The name or title of the document</t>
+          <t>Brief description of what the document contains</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -748,7 +752,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -767,23 +771,23 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Document types[]</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Brief description of what the document contains</t>
+          <t>List of codelist references that the document covers</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -802,18 +806,18 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Document types[]</t>
+          <t>Uploaded date</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>List of codelist references that the document covers</t>
+          <t>The date the document was uploaded to the application</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -837,23 +841,27 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Uploaded date</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Base64</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>The date the document was uploaded to the application</t>
+          <t>Base64-encoded content of the file for inline file uploads</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -877,12 +885,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Base64</t>
+          <t>Filename</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Base64-encoded content of the file for inline file uploads</t>
+          <t>Name of the file being uploaded</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -892,7 +900,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -916,12 +924,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Filename</t>
+          <t>MIME type</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Name of the file being uploaded</t>
+          <t>The file's MIME type such as application/pdf or image/jpeg</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -931,7 +939,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -955,17 +963,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>MIME type</t>
+          <t>File size</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>The file's MIME type such as application/pdf or image/jpeg</t>
+          <t>Size of the file in bytes that can be used to enforce limits</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -984,22 +992,18 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Documents[]</t>
+          <t>Fee</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>File size</t>
-        </is>
-      </c>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Size of the file in bytes that can be used to enforce limits</t>
+          <t>The total amount due for the application fee</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1009,7 +1013,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1028,13 +1032,13 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Amount paid</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>The total amount due for the application fee</t>
+          <t>The amount paid towards the application fee</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1063,75 +1067,67 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Amount paid</t>
+          <t>Transactions[]</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>The amount paid towards the application fee</t>
+          <t>References to payments or financial transactions related to this application</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Advertisement location</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Where the advertisement being applied to be built will be located</t>
+        </is>
+      </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Fee</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Transactions[]</t>
-        </is>
-      </c>
+          <t>Is advert in place</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>References to payments or financial transactions related to this application</t>
+          <t>Whether the advertisement is already in place</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Advertisement location</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Where the advertisement being applied to be built will be located</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Is advert in place</t>
+          <t>Advert placed date</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -1139,17 +1135,17 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Whether the advertisement is already in place</t>
+          <t>Date when the advertisement was placed (YYYY-MM-DD format)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1154,7 @@
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Advert placed date</t>
+          <t>Is replacement advert</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1166,17 +1162,17 @@
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Date when the advertisement was placed (YYYY-MM-DD format)</t>
+          <t>Whether this is a replacement advertisement</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1185,20 +1181,24 @@
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Is replacement advert</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
+          <t>Document reference[]</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Whether this is a replacement advertisement</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1212,24 +1212,20 @@
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Document reference[]</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
+          <t>Is advert overhanging</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>Whether the advertisement will project over a footpath or other public highway</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1239,11 +1235,19 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Advert period</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>How long the proposed advertisement will be shown.</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Is advert overhanging</t>
+          <t>Advert start date</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -1251,12 +1255,12 @@
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Whether the advertisement will project over a footpath or other public highway</t>
+          <t>The start of the time period that consent to advertisement is sought</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1266,19 +1270,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Advert period</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>How long the proposed advertisement will be shown.</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Advert start date</t>
+          <t>Advert end date</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -1286,7 +1282,7 @@
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>The start of the time period that consent to advertisement is sought</t>
+          <t>The end of the time period that consent to advertisement is sought</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1301,11 +1297,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Advertisement types</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>What type of advertisements are proposed and how many there will be.</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Advert end date</t>
+          <t>Advertisement proposal description</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -1313,12 +1317,12 @@
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>The end of the time period that consent to advertisement is sought</t>
+          <t>Description of the advertisement proposal</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1328,32 +1332,28 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Advertisement types</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>What type of advertisements are proposed and how many there will be.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Advertisement proposal description</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>Advertisement proposal type[]</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Advertisement type</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Description of the advertisement proposal</t>
+          <t>One of the advertisement-types or other</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1372,19 +1372,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Advertisement type</t>
+          <t>Advertisement count</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>One of the advertisement-types or other</t>
+          <t>Number of this type of advertisement</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1403,45 +1403,49 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Advertisement count</t>
+          <t>Advertisement other description</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Number of this type of advertisement</t>
+          <t>Details required if other advertisement type is selected</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Agent contact details</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information if an agent is being used.</t>
+        </is>
+      </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Advertisement proposal type[]</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Advertisement other description</t>
-        </is>
-      </c>
+          <t>Agent reference</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Details required if other advertisement type is selected</t>
+          <t>A reference to an agent object</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1451,32 +1455,28 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Agent contact details</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information if an agent is being used.</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Agent reference</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
+          <t>Contact details</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>A reference to an agent object</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1500,14 +1500,18 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr"/>
+          <t>Phone number(s)[]</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Phone number</t>
+        </is>
+      </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1517,7 +1521,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1536,18 +1540,18 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Contact priority</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The priority of a number</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -1557,51 +1561,47 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Agent details</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information if an agent is being used.</t>
+        </is>
+      </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Contact details</t>
+          <t>agent</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Phone number(s)[]</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Contact priority</t>
-        </is>
-      </c>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>The priority of a number</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Agent details</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information if an agent is being used.</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
           <t>agent</t>
@@ -1609,14 +1609,18 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>The title of the individual</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1626,7 +1630,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1645,13 +1649,13 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>The title of the individual</t>
+          <t>The first name of the individual</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1661,7 +1665,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1680,13 +1684,13 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>The first name of the individual</t>
+          <t>The last name of the individual</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1715,13 +1719,13 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>The last name of the individual</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1750,13 +1754,13 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -1766,7 +1770,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1780,18 +1784,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Postcode</t>
-        </is>
-      </c>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>The name of a company (that the agent works for)</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1815,19 +1815,19 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>User role</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>The name of a company (that the agent works for)</t>
+          <t>The role of the named individual. Agent or proxy</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -1837,58 +1837,58 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Applicant contact details</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Telephone number and email address of the applicant.</t>
+        </is>
+      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>User role</t>
-        </is>
-      </c>
+          <t>Applicant reference</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>The role of the named individual. Agent or proxy</t>
+          <t>Reference to match contact details to a named individual from the applicant details component</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Applicant contact details</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Telephone number and email address of the applicant.</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Applicant reference</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>Contact details</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Reference to match contact details to a named individual from the applicant details component</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -1912,14 +1912,18 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
+          <t>Phone number(s)[]</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Phone number</t>
+        </is>
+      </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -1929,7 +1933,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1948,18 +1952,18 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Contact priority</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The priority of a number</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -1969,51 +1973,47 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Applicant details</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information for the parties making the application.</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Contact details</t>
+          <t>Applicants[]</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Phone number(s)[]</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Contact priority</t>
-        </is>
-      </c>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>The priority of a number</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Applicant details</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information for the parties making the application.</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Applicants[]</t>
@@ -2021,14 +2021,18 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>The title of the individual</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2038,7 +2042,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2057,13 +2061,13 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>The title of the individual</t>
+          <t>The first name of the individual</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2073,7 +2077,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2092,13 +2096,13 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>The first name of the individual</t>
+          <t>The last name of the individual</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2127,13 +2131,13 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>The last name of the individual</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2162,13 +2166,13 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2178,32 +2182,32 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Checking whether all the requirements of the form have been met, such as proof of payment or supporting documentation.</t>
+        </is>
+      </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Applicants[]</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Postcode</t>
-        </is>
-      </c>
+          <t>National requirement types[]</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>List of the document types required for the given application type</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2213,24 +2217,24 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Community consultation</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Checking whether all the requirements of the form have been met, such as proof of payment or supporting documentation.</t>
+          <t>What community consultation activities have taken place as part of the application</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>National requirement types[]</t>
+          <t>Have consulted</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -2238,12 +2242,12 @@
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>List of the document types required for the given application type</t>
+          <t>Whether community consultation has been carried out</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -2253,19 +2257,11 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Community consultation</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>What community consultation activities have taken place as part of the application</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Have consulted</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
@@ -2273,26 +2269,34 @@
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Whether community consultation has been carried out</t>
+          <t>Provide details of the community consultation</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Conflict of interest</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
+        </is>
+      </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Conflict to declare</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -2300,34 +2304,26 @@
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Provide details of the community consultation</t>
+          <t>Indicates whether any named applicant or agent has a relationship to the planning authority that must be declared</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Conflict of interest</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
-        </is>
-      </c>
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Conflict to declare</t>
+          <t>Conflict person name</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -2335,17 +2331,17 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Indicates whether any named applicant or agent has a relationship to the planning authority that must be declared</t>
+          <t>Name of the individual with the conflict of interest that matches one of the names provided in applicants/agent section</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2350,7 @@
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Conflict person name</t>
+          <t>Conflict details</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -2362,7 +2358,7 @@
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Name of the individual with the conflict of interest that matches one of the names provided in applicants/agent section</t>
+          <t>Details of the conflict of interest including name, role and how the individual is related to the planning authority</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2377,11 +2373,19 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Interest in land</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Whether the applicant owns or has permission to use the land where the proposed advertisement will be placed</t>
+        </is>
+      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Conflict details</t>
+          <t>Applicant owns land</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -2389,34 +2393,26 @@
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Details of the conflict of interest including name, role and how the individual is related to the planning authority</t>
+          <t>True or False indicating whether the applicant owns the land where the advertisement will be displayed</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Interest in land</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Whether the applicant owns or has permission to use the land where the proposed advertisement will be placed</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Applicant owns land</t>
+          <t>Permission obtained</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -2424,7 +2420,7 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>True or False indicating whether the applicant owns the land where the advertisement will be displayed</t>
+          <t>True or False indicating whether permission of the owner for the display of an advertisement has been obtained</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2434,7 +2430,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2439,7 @@
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Permission obtained</t>
+          <t>Permission not obtained details</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -2451,12 +2447,12 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>True or False indicating whether permission of the owner for the display of an advertisement has been obtained</t>
+          <t>Details explaining why permission from the land owner has not been obtained for the advertisement display</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -2466,11 +2462,19 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Declaration</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Signed and dated verification of the application's accuracy.</t>
+        </is>
+      </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Permission not obtained details</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -2478,7 +2482,7 @@
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Details explaining why permission from the land owner has not been obtained for the advertisement display</t>
+          <t>A name of a person</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -2488,24 +2492,16 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Declaration</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Signed and dated verification of the application's accuracy.</t>
-        </is>
-      </c>
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Declaration confirmed</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr"/>
@@ -2513,12 +2509,12 @@
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>A name of a person</t>
+          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -2532,7 +2528,7 @@
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Declaration confirmed</t>
+          <t>Declaration date</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
@@ -2540,12 +2536,12 @@
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
+          <t>The date the declaration was made</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -2555,11 +2551,19 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Pre-application advice</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Details of pre-application advice previously received from the planning authority</t>
+        </is>
+      </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Declaration date</t>
+          <t>Pre-application advice sought</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
@@ -2567,12 +2571,12 @@
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>The date the declaration was made</t>
+          <t>Whether pre-application advice has been sought from the planning authority</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -2582,19 +2586,11 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Pre-application advice</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Details of pre-application advice previously received from the planning authority</t>
-        </is>
-      </c>
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Pre-application advice sought</t>
+          <t>Officer name</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr"/>
@@ -2602,17 +2598,17 @@
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Whether pre-application advice has been sought from the planning authority</t>
+          <t>Name of the planning officer who provided the pre-application advice</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2617,7 @@
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Officer name</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
@@ -2629,7 +2625,7 @@
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Name of the planning officer who provided the pre-application advice</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -2648,7 +2644,7 @@
       <c r="B67" s="2" t="n"/>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Advice date</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr"/>
@@ -2656,7 +2652,7 @@
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -2675,7 +2671,7 @@
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Advice date</t>
+          <t>Advice summary</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
@@ -2683,7 +2679,7 @@
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
+          <t>Summary of the pre-application advice received from the planning authority</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -2698,24 +2694,36 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Proposed advert details</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Details of the proposed advertisements such as their size and how they are made</t>
+        </is>
+      </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Advice summary</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr"/>
+          <t>Advertisements[]</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Height from ground</t>
+        </is>
+      </c>
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Summary of the pre-application advice received from the planning authority</t>
+          <t>Height, in metres, from ground to the base of the advertisement</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -2725,16 +2733,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Proposed advert details</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Details of the proposed advertisements such as their size and how they are made</t>
-        </is>
-      </c>
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Advertisements[]</t>
@@ -2742,14 +2742,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Height from ground</t>
+          <t>Height</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Height, in metres, from ground to the base of the advertisement</t>
+          <t>Height, in metres, of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -2773,14 +2773,14 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Height</t>
+          <t>Width</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Height, in metres, of dimensions of advertisement</t>
+          <t>Width of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -2804,14 +2804,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Width</t>
+          <t>Depth</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Width of dimensions of advertisement</t>
+          <t>Depth, in metres, of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -2835,14 +2835,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Depth</t>
+          <t>Symbol height max</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Depth, in metres, of dimensions of advertisement</t>
+          <t>Maximum height, in metres, of any individual letters or symbols</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -2866,19 +2866,19 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Symbol height max</t>
+          <t>Colour</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Maximum height, in metres, of any individual letters or symbols</t>
+          <t>Colour of proposed sign</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -2897,14 +2897,14 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Colour of proposed sign</t>
+          <t>Materials of proposed sign</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -2928,19 +2928,19 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Max projection</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Materials of proposed sign</t>
+          <t>Maximum projection, in metres, of the advertisement from the face of the building</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -2959,19 +2959,19 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Max projection</t>
+          <t>Illuminated</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Maximum projection, in metres, of the advertisement from the face of the building</t>
+          <t>Will the sign(s) be illuminated?</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -2990,19 +2990,19 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Illuminated</t>
+          <t>Illumination method</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Will the sign(s) be illuminated?</t>
+          <t>Method of illumination for the advertisement</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3021,19 +3021,19 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Illumination method</t>
+          <t>Illuminance level</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Method of illumination for the advertisement</t>
+          <t>Level of illuminance for the advertisement</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Illuminance level</t>
+          <t>Illumination type</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Level of illuminance for the advertisement</t>
+          <t>Type of illumination (static or intermittent)</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -3074,28 +3074,36 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n"/>
-      <c r="B81" s="2" t="n"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Site details</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Where the proposed development will be built.</t>
+        </is>
+      </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Advertisements[]</t>
+          <t>Site locations[]</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Illumination type</t>
+          <t>Site boundary</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Type of illumination (static or intermittent)</t>
+          <t>Geometry of the site of the development, typically in GeoJSON format</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>wkt</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -3105,16 +3113,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Site details</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>Where the proposed development will be built.</t>
-        </is>
-      </c>
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Site locations[]</t>
@@ -3122,19 +3122,19 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Site boundary</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Geometry of the site of the development, typically in GeoJSON format</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>wkt</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -3153,14 +3153,14 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -3184,19 +3184,19 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Easting</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -3215,14 +3215,14 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Easting</t>
+          <t>Northing</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
+          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -3246,14 +3246,14 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Northing</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
+          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -3277,14 +3277,14 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -3308,19 +3308,19 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>A text description providing details about the subject. For parking changes, this describes how the proposed works affect existing car parking arrangements.</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -3339,14 +3339,14 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>UPRNs[]</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>A text description providing details about the subject. For parking changes, this describes how the proposed works affect existing car parking arrangements.</t>
+          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -3361,50 +3361,46 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n"/>
-      <c r="B90" s="2" t="n"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Site Visit Details</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Information to help the planning authority arrange a site visit</t>
+        </is>
+      </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>UPRNs[]</t>
-        </is>
-      </c>
+          <t>Site seen from public area</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
+          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>Site Visit Details</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>Information to help the planning authority arrange a site visit</t>
-        </is>
-      </c>
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="n"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Site seen from public area</t>
+          <t>Site visit contact type</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr"/>
@@ -3412,12 +3408,12 @@
       <c r="F91" s="2" t="inlineStr"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
+          <t>Indicates who the authority should contact to arrange a site visit</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -3431,7 +3427,7 @@
       <c r="B92" s="2" t="n"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Site visit contact type</t>
+          <t>Contact reference</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr"/>
@@ -3439,17 +3435,17 @@
       <c r="F92" s="2" t="inlineStr"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Indicates who the authority should contact to arrange a site visit</t>
+          <t>The reference of the applicant or agent who should be contacted for site visits</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -3458,15 +3454,19 @@
       <c r="B93" s="2" t="n"/>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Contact reference</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr"/>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Full name</t>
+        </is>
+      </c>
       <c r="E93" s="2" t="inlineStr"/>
       <c r="F93" s="2" t="inlineStr"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>The reference of the applicant or agent who should be contacted for site visits</t>
+          <t>The complete name of a person</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3490,14 +3490,14 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Full name</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>The complete name of a person</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -3521,14 +3521,14 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -3537,37 +3537,6 @@
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="n"/>
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr"/>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
@@ -3575,40 +3544,40 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A35:A42"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="B35:B42"/>
-    <mergeCell ref="A53"/>
-    <mergeCell ref="B91:B96"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B82:B90"/>
-    <mergeCell ref="A20:A24"/>
-    <mergeCell ref="A2:A19"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="B47:B52"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="B43:B46"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B20:B24"/>
-    <mergeCell ref="B56:B58"/>
-    <mergeCell ref="B59:B61"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="A70:A81"/>
-    <mergeCell ref="A91:A96"/>
-    <mergeCell ref="A82:A90"/>
-    <mergeCell ref="A47:A52"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B70:B81"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A43:A46"/>
-    <mergeCell ref="B53"/>
-    <mergeCell ref="A65:A69"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B2:B19"/>
-    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A34:A41"/>
+    <mergeCell ref="A52"/>
+    <mergeCell ref="B19:B23"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B2:B18"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="A69:A80"/>
+    <mergeCell ref="A19:A23"/>
+    <mergeCell ref="A81:A89"/>
+    <mergeCell ref="A64:A68"/>
+    <mergeCell ref="A90:A95"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="B52"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A46:A51"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A2:A18"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A61:A63"/>
+    <mergeCell ref="B81:B89"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B34:B41"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B69:B80"/>
+    <mergeCell ref="A55:A57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Latest generated outputs 2026-04-21
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/advertising-advertising.xlsx
+++ b/generated/spreadsheet/advertising-advertising.xlsx
@@ -2541,7 +2541,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">

</xml_diff>